<commit_message>
updated run.bat and modified DDT Tc
</commit_message>
<xml_diff>
--- a/testdata/data_for_registration.xlsx
+++ b/testdata/data_for_registration.xlsx
@@ -51,21 +51,9 @@
     <t>Male</t>
   </si>
   <si>
-    <t>password@123</t>
-  </si>
-  <si>
     <t>pass</t>
   </si>
   <si>
-    <t>chintu</t>
-  </si>
-  <si>
-    <t>vangdu</t>
-  </si>
-  <si>
-    <t>chintu@yahoo.com</t>
-  </si>
-  <si>
     <t>Engineer</t>
   </si>
   <si>
@@ -90,13 +78,25 @@
     <t>fail</t>
   </si>
   <si>
-    <t>tiku</t>
-  </si>
-  <si>
-    <t>miku</t>
-  </si>
-  <si>
-    <t>tikumiku@gmail.com</t>
+    <t>Vikram</t>
+  </si>
+  <si>
+    <t>Password@123</t>
+  </si>
+  <si>
+    <t>Rajeev</t>
+  </si>
+  <si>
+    <t>Jagdish</t>
+  </si>
+  <si>
+    <t>rajeevj@gmail.com</t>
+  </si>
+  <si>
+    <t>Pillai</t>
+  </si>
+  <si>
+    <t>vikramp@yahoo.com</t>
   </si>
 </sst>
 </file>
@@ -485,13 +485,13 @@
     </row>
     <row r="2" spans="1:9">
       <c r="A2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>24</v>
-      </c>
-      <c r="B2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>26</v>
       </c>
       <c r="D2">
         <v>1234098760</v>
@@ -503,59 +503,59 @@
         <v>10</v>
       </c>
       <c r="G2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="I2" t="s">
         <v>11</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="I2" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:9">
       <c r="A3" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="D3">
         <v>9876123450</v>
       </c>
       <c r="E3" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F3" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="I3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:9">
       <c r="A4" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="B4" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D4">
         <v>1234567890</v>
       </c>
       <c r="E4" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="F4" t="s">
         <v>10</v>
@@ -567,18 +567,18 @@
         <v>1</v>
       </c>
       <c r="I4" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="C2" r:id="rId1"/>
     <hyperlink ref="G2" r:id="rId2"/>
-    <hyperlink ref="H2" r:id="rId3"/>
-    <hyperlink ref="C3" r:id="rId4"/>
-    <hyperlink ref="G3" r:id="rId5"/>
-    <hyperlink ref="H3" r:id="rId6"/>
-    <hyperlink ref="C4" r:id="rId7"/>
+    <hyperlink ref="C3" r:id="rId3"/>
+    <hyperlink ref="G3" r:id="rId4"/>
+    <hyperlink ref="H3" r:id="rId5"/>
+    <hyperlink ref="C4" r:id="rId6"/>
+    <hyperlink ref="H2" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>